<commit_message>
added new log and changed mecamh tags
</commit_message>
<xml_diff>
--- a/SurveyQuestions/outputs/MECAMH_question_score.xlsx
+++ b/SurveyQuestions/outputs/MECAMH_question_score.xlsx
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>[State] Anxiety (modelled on the STAI)</t>
+          <t>Anxiety</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Anticipatory Traumatic Reaction – Feelings Sub-Scale (Hopwood et al. 2017)</t>
+          <t>Anticipatory Traumatic Reaction</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Coping Responses (Ojala 2012)</t>
+          <t>Coping Responses</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Climate Change Worry (Ojala 2012)</t>
+          <t>Climate Change Worry</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">

</xml_diff>